<commit_message>
Fix concatenated price numbers in The Henley I 2座 8A/9A and 壹沐第2期 Excel and web data files
</commit_message>
<xml_diff>
--- a/files/九龙-启德-The Henley I.xlsx
+++ b/files/九龙-启德-The Henley I.xlsx
@@ -14313,10 +14313,10 @@
         </is>
       </c>
       <c r="H221" s="5" t="n">
-        <v>1837500018651000</v>
+        <v>18651000</v>
       </c>
       <c r="I221" s="5" t="n">
-        <v>3365384649544</v>
+        <v>34160</v>
       </c>
       <c r="J221" s="3" t="inlineStr">
         <is>
@@ -14324,10 +14324,10 @@
         </is>
       </c>
       <c r="K221" s="5" t="n">
-        <v>1697827048483200</v>
+        <v>17233524</v>
       </c>
       <c r="L221" s="5" t="n">
-        <v>3109573348870</v>
+        <v>31563</v>
       </c>
       <c r="M221" s="3" t="inlineStr">
         <is>
@@ -15615,10 +15615,10 @@
         </is>
       </c>
       <c r="H242" s="5" t="n">
-        <v>2796300028662000</v>
+        <v>28662000</v>
       </c>
       <c r="I242" s="5" t="n">
-        <v>3145444351701</v>
+        <v>32241</v>
       </c>
       <c r="J242" s="3" t="inlineStr">
         <is>
@@ -15626,10 +15626,10 @@
         </is>
       </c>
       <c r="K242" s="5" t="n">
-        <v>2583746272733300</v>
+        <v>26483688</v>
       </c>
       <c r="L242" s="5" t="n">
-        <v>2906351262917</v>
+        <v>29790</v>
       </c>
       <c r="M242" s="3" t="inlineStr">
         <is>
@@ -15987,10 +15987,10 @@
         </is>
       </c>
       <c r="H248" s="5" t="n">
-        <v>1803600018307000</v>
+        <v>18307000</v>
       </c>
       <c r="I248" s="5" t="n">
-        <v>3303296736826</v>
+        <v>33529</v>
       </c>
       <c r="J248" s="3" t="inlineStr">
         <is>
@@ -15998,10 +15998,10 @@
         </is>
       </c>
       <c r="K248" s="5" t="n">
-        <v>1666503871915300</v>
+        <v>16915668</v>
       </c>
       <c r="L248" s="5" t="n">
-        <v>3052204893618</v>
+        <v>30981</v>
       </c>
       <c r="M248" s="3" t="inlineStr">
         <is>
@@ -16173,10 +16173,10 @@
         </is>
       </c>
       <c r="H251" s="5" t="n">
-        <v>2796000028659000</v>
+        <v>28659000</v>
       </c>
       <c r="I251" s="5" t="n">
-        <v>3145106893880</v>
+        <v>32237</v>
       </c>
       <c r="J251" s="3" t="inlineStr">
         <is>
@@ -16184,10 +16184,10 @@
         </is>
       </c>
       <c r="K251" s="5" t="n">
-        <v>2583469076480500</v>
+        <v>26480916</v>
       </c>
       <c r="L251" s="5" t="n">
-        <v>2906039456109</v>
+        <v>29787</v>
       </c>
       <c r="M251" s="3" t="inlineStr">
         <is>
@@ -16545,10 +16545,10 @@
         </is>
       </c>
       <c r="H257" s="5" t="n">
-        <v>1797900018249000</v>
+        <v>18249000</v>
       </c>
       <c r="I257" s="5" t="n">
-        <v>3292857176280</v>
+        <v>33423</v>
       </c>
       <c r="J257" s="3" t="inlineStr">
         <is>
@@ -16556,10 +16556,10 @@
         </is>
       </c>
       <c r="K257" s="5" t="n">
-        <v>1661237143111700</v>
+        <v>16862076</v>
       </c>
       <c r="L257" s="5" t="n">
-        <v>3042558870168</v>
+        <v>30883</v>
       </c>
       <c r="M257" s="3" t="inlineStr">
         <is>
@@ -32663,8 +32663,8 @@
       <c r="B31" s="24" t="inlineStr">
         <is>
           <t>A | 889呎 (3房)
-$279630002866万
-$3,145,444,351,701/呎
+万
+,241/呎
 (暂停销售)</t>
         </is>
       </c>

</xml_diff>